<commit_message>
Optimize RBFNN benchmark MAPE results
</commit_message>
<xml_diff>
--- a/optimized_version/metadata/benchmark_metrics/optimized_benchmark_validation_testing_metrics.xlsx
+++ b/optimized_version/metadata/benchmark_metrics/optimized_benchmark_validation_testing_metrics.xlsx
@@ -527,28 +527,28 @@
         <v>29</v>
       </c>
       <c r="D3" t="n">
-        <v>3.434675445626739</v>
+        <v>3.451840791241192</v>
       </c>
       <c r="E3" t="n">
-        <v>1.709227388475206</v>
+        <v>1.71664344441512</v>
       </c>
       <c r="F3" t="n">
-        <v>2.759805153519004</v>
+        <v>2.769457742259154</v>
       </c>
       <c r="G3" t="n">
-        <v>0.9288569267050834</v>
+        <v>0.9283584018428611</v>
       </c>
       <c r="H3" t="n">
-        <v>3.547024793233517</v>
+        <v>3.572705810229515</v>
       </c>
       <c r="I3" t="n">
-        <v>1.89576248035897</v>
+        <v>1.928287727407958</v>
       </c>
       <c r="J3" t="n">
-        <v>3.476679847242576</v>
+        <v>3.507520889972095</v>
       </c>
       <c r="K3" t="n">
-        <v>0.8967093208080847</v>
+        <v>0.8948686441752667</v>
       </c>
     </row>
     <row r="4">
@@ -581,13 +581,13 @@
         <v>2.161182022518592</v>
       </c>
       <c r="I4" t="n">
-        <v>1.933811975752545</v>
+        <v>1.933811975752544</v>
       </c>
       <c r="J4" t="n">
         <v>5.005367101266894</v>
       </c>
       <c r="K4" t="n">
-        <v>0.9047764040971429</v>
+        <v>0.904776404097143</v>
       </c>
     </row>
     <row r="5">
@@ -605,28 +605,28 @@
         <v>30</v>
       </c>
       <c r="D5" t="n">
-        <v>1.720696696292816</v>
+        <v>1.744494832966965</v>
       </c>
       <c r="E5" t="n">
-        <v>1.592372721660347</v>
+        <v>1.620137456758978</v>
       </c>
       <c r="F5" t="n">
-        <v>4.182296397495707</v>
+        <v>4.236730177584649</v>
       </c>
       <c r="G5" t="n">
-        <v>0.8311074489061773</v>
+        <v>0.8266824694896371</v>
       </c>
       <c r="H5" t="n">
-        <v>2.533877892844516</v>
+        <v>2.553581038972992</v>
       </c>
       <c r="I5" t="n">
-        <v>2.126042828874627</v>
+        <v>2.173190188862365</v>
       </c>
       <c r="J5" t="n">
-        <v>5.248554229849789</v>
+        <v>5.219189186025636</v>
       </c>
       <c r="K5" t="n">
-        <v>0.8952986971951848</v>
+        <v>0.8964670027188831</v>
       </c>
     </row>
     <row r="6">
@@ -644,10 +644,10 @@
         <v>30</v>
       </c>
       <c r="D6" t="n">
-        <v>1.774556659412655</v>
+        <v>1.774556659412656</v>
       </c>
       <c r="E6" t="n">
-        <v>1.456443027139063</v>
+        <v>1.456443027139064</v>
       </c>
       <c r="F6" t="n">
         <v>3.980111616750163</v>
@@ -656,13 +656,13 @@
         <v>0.9338717637429117</v>
       </c>
       <c r="H6" t="n">
-        <v>1.164311265066938</v>
+        <v>1.164311265066937</v>
       </c>
       <c r="I6" t="n">
         <v>1.365183498334776</v>
       </c>
       <c r="J6" t="n">
-        <v>3.45407003146723</v>
+        <v>3.454070031467231</v>
       </c>
       <c r="K6" t="n">
         <v>0.9311114849194968</v>
@@ -683,28 +683,28 @@
         <v>30</v>
       </c>
       <c r="D7" t="n">
-        <v>1.631781368537392</v>
+        <v>1.71745827658513</v>
       </c>
       <c r="E7" t="n">
-        <v>1.352547138398912</v>
+        <v>1.382999808041294</v>
       </c>
       <c r="F7" t="n">
-        <v>3.766868353845349</v>
+        <v>3.902914547977252</v>
       </c>
       <c r="G7" t="n">
-        <v>0.9407678738806523</v>
+        <v>0.9364120941983439</v>
       </c>
       <c r="H7" t="n">
-        <v>1.071541685667849</v>
+        <v>1.05126148122372</v>
       </c>
       <c r="I7" t="n">
-        <v>1.290699641116295</v>
+        <v>1.26574175268856</v>
       </c>
       <c r="J7" t="n">
-        <v>3.229582747393507</v>
+        <v>3.272789934700768</v>
       </c>
       <c r="K7" t="n">
-        <v>0.9397749209248093</v>
+        <v>0.9381526910348479</v>
       </c>
     </row>
     <row r="8">
@@ -734,7 +734,7 @@
         <v>0.9049217652560917</v>
       </c>
       <c r="H8" t="n">
-        <v>4.200484513643535</v>
+        <v>4.200484513643534</v>
       </c>
       <c r="I8" t="n">
         <v>1.598433789599624</v>
@@ -761,28 +761,28 @@
         <v>29</v>
       </c>
       <c r="D9" t="n">
-        <v>4.164354919883476</v>
+        <v>4.180765718437955</v>
       </c>
       <c r="E9" t="n">
-        <v>1.47443636235442</v>
+        <v>1.479533045060711</v>
       </c>
       <c r="F9" t="n">
-        <v>2.18347851957049</v>
+        <v>2.188924444285949</v>
       </c>
       <c r="G9" t="n">
-        <v>0.9083943896883839</v>
+        <v>0.907936863415191</v>
       </c>
       <c r="H9" t="n">
-        <v>4.269387443260273</v>
+        <v>4.227887501466392</v>
       </c>
       <c r="I9" t="n">
-        <v>1.632710428796588</v>
+        <v>1.614116089819198</v>
       </c>
       <c r="J9" t="n">
-        <v>2.244636714582071</v>
+        <v>2.233242150647068</v>
       </c>
       <c r="K9" t="n">
-        <v>0.8955506035042257</v>
+        <v>0.8966083555186281</v>
       </c>
     </row>
     <row r="10">
@@ -800,10 +800,10 @@
         <v>32</v>
       </c>
       <c r="D10" t="n">
-        <v>2.967630624280722</v>
+        <v>2.967630624280723</v>
       </c>
       <c r="E10" t="n">
-        <v>4.534963565508412</v>
+        <v>4.534963565508413</v>
       </c>
       <c r="F10" t="n">
         <v>8.150774218763839</v>
@@ -812,13 +812,13 @@
         <v>0.8278085456100657</v>
       </c>
       <c r="H10" t="n">
-        <v>19.87941386644248</v>
+        <v>19.87941386644245</v>
       </c>
       <c r="I10" t="n">
-        <v>8.033408364487519</v>
+        <v>8.033408364487512</v>
       </c>
       <c r="J10" t="n">
-        <v>12.19846815910363</v>
+        <v>12.19846815910361</v>
       </c>
       <c r="K10" t="n">
         <v>0.9560946692216128</v>
@@ -839,28 +839,28 @@
         <v>32</v>
       </c>
       <c r="D11" t="n">
-        <v>2.691804783297085</v>
+        <v>2.664091660721063</v>
       </c>
       <c r="E11" t="n">
-        <v>4.08534347512202</v>
+        <v>4.047043590636704</v>
       </c>
       <c r="F11" t="n">
-        <v>7.719378035568226</v>
+        <v>7.62303727279962</v>
       </c>
       <c r="G11" t="n">
-        <v>0.8455533517746964</v>
+        <v>0.849384400566642</v>
       </c>
       <c r="H11" t="n">
-        <v>35.33122290805673</v>
+        <v>37.5409989513803</v>
       </c>
       <c r="I11" t="n">
-        <v>13.32873844484557</v>
+        <v>14.05841895127159</v>
       </c>
       <c r="J11" t="n">
-        <v>21.53924194978802</v>
+        <v>22.57904593416176</v>
       </c>
       <c r="K11" t="n">
-        <v>0.8631113347053906</v>
+        <v>0.8495757572901768</v>
       </c>
     </row>
     <row r="12">
@@ -890,7 +890,7 @@
         <v>0.8274916190187004</v>
       </c>
       <c r="H12" t="n">
-        <v>4.294212888621111</v>
+        <v>4.294212888621112</v>
       </c>
       <c r="I12" t="n">
         <v>1.526733463455669</v>
@@ -917,28 +917,28 @@
         <v>29</v>
       </c>
       <c r="D13" t="n">
-        <v>4.074631372425127</v>
+        <v>4.083274772187985</v>
       </c>
       <c r="E13" t="n">
-        <v>1.315960292496638</v>
+        <v>1.314191121949027</v>
       </c>
       <c r="F13" t="n">
-        <v>2.058319755321813</v>
+        <v>2.057274702140808</v>
       </c>
       <c r="G13" t="n">
-        <v>0.8325977597722016</v>
+        <v>0.832767704050032</v>
       </c>
       <c r="H13" t="n">
-        <v>4.306239015112928</v>
+        <v>4.31108012753736</v>
       </c>
       <c r="I13" t="n">
-        <v>1.543080770395224</v>
+        <v>1.542352377302068</v>
       </c>
       <c r="J13" t="n">
-        <v>2.171666227220461</v>
+        <v>2.173520856365352</v>
       </c>
       <c r="K13" t="n">
-        <v>0.9115345919289649</v>
+        <v>0.9113834263574155</v>
       </c>
     </row>
   </sheetData>

</xml_diff>